<commit_message>
Tracker: original seed 1 R1 done / R2 ep 69 (val 0.878); smoke test confirms backbone fix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experiment_Tracker_X1X2.xlsx
+++ b/experiments/Experiment_Tracker_X1X2.xlsx
@@ -594,7 +594,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2)</t>
+          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2) · อัปเดต 2026-10-02 10:45</t>
         </is>
       </c>
     </row>
@@ -942,13 +942,13 @@
         </is>
       </c>
       <c r="I8" s="6" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>200</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="L8" s="6" t="n">
         <v>200</v>
@@ -958,7 +958,7 @@
         <v/>
       </c>
       <c r="N8" s="8" t="n">
-        <v>0.654</v>
+        <v>0.878</v>
       </c>
       <c r="O8" s="9">
         <f>IF(D8="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C8)*(Results!$B$5:$B$50=D8)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
@@ -976,7 +976,7 @@
       <c r="R8" s="6" t="inlineStr"/>
       <c r="S8" s="10" t="inlineStr">
         <is>
-          <t>ep 1 val_acc 0.654 = ทาย Normal ทั้งหมด (ปกติของ R1)</t>
+          <t>10-02 10:45: R1 เสร็จ (val 0.7195), R2 ep 69 val 0.878 · ~4 นาที/epoch</t>
         </is>
       </c>
     </row>
@@ -1644,17 +1644,17 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>กำลังรัน</t>
+          <t>เสร็จ</t>
         </is>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J19" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>3</v>
@@ -1663,7 +1663,9 @@
         <f>IFERROR((I19+K19)/(J19+L19),"")</f>
         <v/>
       </c>
-      <c r="N19" s="8" t="n"/>
+      <c r="N19" s="8" t="n">
+        <v>0.6921</v>
+      </c>
       <c r="O19" s="9">
         <f>IF(D19="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C19)*(Results!$B$5:$B$50=D19)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
         <v/>
@@ -1674,13 +1676,17 @@
       </c>
       <c r="Q19" s="6" t="inlineStr">
         <is>
-          <t>2026-10-01 17:00</t>
-        </is>
-      </c>
-      <c r="R19" s="6" t="inlineStr"/>
+          <t>2026-10-01 16:55</t>
+        </is>
+      </c>
+      <c r="R19" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="S19" s="10" t="inlineStr">
         <is>
-          <t>ไม่นับเป็นผล</t>
+          <t>R1 0.654 → R2 0.692 &gt; 0.654 ✓ แก้ backbone สำเร็จ · ไม่นับเป็นผล</t>
         </is>
       </c>
     </row>
@@ -3452,25 +3458,73 @@
       <c r="E10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="4" t="n"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>smoke test เสร็จ: R2 val_acc 0.692 (&gt; 0.654)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>ยืนยันว่าแก้ bug backbone สำเร็จ</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="4" t="n"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>R1 เสร็จ val 0.7195; R2 ep 69/200 val 0.878 — original ไม่ collapse แล้ว</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>GPU 1 ว่างตั้งแต่ smoke test จบ</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="4" t="n"/>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>ตั้ง SSH key Mac → เครื่อง 29 (แก้ permission ~/.ssh)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Claude เช็คสถานะเองได้</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>

</xml_diff>

<commit_message>
Tracker: start unlearned seeds 2-3 on GPU 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experiment_Tracker_X1X2.xlsx
+++ b/experiments/Experiment_Tracker_X1X2.xlsx
@@ -1144,11 +1144,17 @@
           <t>unlearn B4-B7 ep50 → USAI R1 → R2 Block5a-B7</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>unlearned</t>
+        </is>
+      </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>ยังไม่เริ่ม</t>
+          <t>กำลังรัน</t>
         </is>
       </c>
       <c r="I11" s="6" t="n">
@@ -1176,9 +1182,17 @@
         <f>IF(D11="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C11)*(Results!$B$5:$B$50=D11)*(Results!$C$5:$C$50="field"),0),0))),""))</f>
         <v/>
       </c>
-      <c r="Q11" s="6" t="inlineStr"/>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-02 10:49</t>
+        </is>
+      </c>
       <c r="R11" s="6" t="inlineStr"/>
-      <c r="S11" s="10" t="inlineStr"/>
+      <c r="S11" s="10" t="inlineStr">
+        <is>
+          <t>~4 นาที/epoch</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1204,8 +1218,14 @@
           <t>unlearn B4-B7 ep50 → USAI R1 → R2 Block5a-B7</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>unlearned</t>
+        </is>
+      </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
           <t>ยังไม่เริ่ม</t>
@@ -1238,7 +1258,11 @@
       </c>
       <c r="Q12" s="6" t="inlineStr"/>
       <c r="R12" s="6" t="inlineStr"/>
-      <c r="S12" s="10" t="inlineStr"/>
+      <c r="S12" s="10" t="inlineStr">
+        <is>
+          <t>ต่อจาก U2 อัตโนมัติ</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -3511,27 +3535,43 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>U2–U3</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>เริ่ม unlearned seed 2 → 3 บน GPU 1 (screen unlearned)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>10:49</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>ตั้ง SSH key Mac → เครื่อง 29 (แก้ permission ~/.ssh)</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Claude เช็คสถานะเองได้</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="4" t="n"/>
+      <c r="E14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>

</xml_diff>

<commit_message>
Tracker: C2 pre-train running on machine 28 (bs 16); GPU 1 of machine 29 fan failure
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experiment_Tracker_X1X2.xlsx
+++ b/experiments/Experiment_Tracker_X1X2.xlsx
@@ -594,7 +594,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2) · อัปเดต 2026-10-02 10:45</t>
+          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2) · อัปเดต 2026-10-02 15:50</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       <c r="D5" s="4" t="inlineStr"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>mini-ImageNet R1 FC · lr 1e-5 · bs 16</t>
+          <t>mini-ImageNet R1 FC · lr 1e-5 · bs 16 · เครื่อง 28 (3090 Ti)</t>
         </is>
       </c>
       <c r="F5" s="6" t="n">
@@ -729,12 +729,12 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>c2_pretrain</t>
+          <t>c2_pretrain (m28)</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>รอตัดสินใจ</t>
+          <t>กำลังรัน</t>
         </is>
       </c>
       <c r="I5" s="6" t="n">
@@ -764,17 +764,13 @@
       </c>
       <c r="Q5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-01 16:42</t>
-        </is>
-      </c>
-      <c r="R5" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-01 16:43</t>
-        </is>
-      </c>
+          <t>2026-10-02 15:49</t>
+        </is>
+      </c>
+      <c r="R5" s="6" t="inlineStr"/>
       <c r="S5" s="10" t="inlineStr">
         <is>
-          <t>OOM ที่ bs 16 บน 2080 Ti → รอ D1</t>
+          <t>~42 นาที/epoch → R1 ≈ 5.8 วัน · เครื่อง 29 OOM (bs 16/8) จึงย้ายมาเครื่อง 28</t>
         </is>
       </c>
     </row>
@@ -797,11 +793,17 @@
       <c r="D6" s="4" t="inlineStr"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>mini-ImageNet R2 unfreeze B4-B7 · lr 1e-6 · bs 16</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
+          <t>mini-ImageNet R2 unfreeze B4-B7 · lr 1e-6 · bs 16 · เครื่อง 28</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>c2_pretrain (m28)</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
           <t>ยังไม่เริ่ม</t>
@@ -836,7 +838,7 @@
       <c r="R6" s="6" t="inlineStr"/>
       <c r="S6" s="10" t="inlineStr">
         <is>
-          <t>ต่อจาก P1</t>
+          <t>ต่อจาก P1 อัตโนมัติ · เสร็จแล้ว copy โมเดลไปเครื่อง 29</t>
         </is>
       </c>
     </row>
@@ -948,7 +950,7 @@
         <v>200</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>69</v>
+        <v>127</v>
       </c>
       <c r="L8" s="6" t="n">
         <v>200</v>
@@ -958,7 +960,7 @@
         <v/>
       </c>
       <c r="N8" s="8" t="n">
-        <v>0.878</v>
+        <v>0.883</v>
       </c>
       <c r="O8" s="9">
         <f>IF(D8="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C8)*(Results!$B$5:$B$50=D8)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
@@ -976,7 +978,7 @@
       <c r="R8" s="6" t="inlineStr"/>
       <c r="S8" s="10" t="inlineStr">
         <is>
-          <t>10-02 10:45: R1 เสร็จ (val 0.7195), R2 ep 69 val 0.878 · ~4 นาที/epoch</t>
+          <t>10-02 15:00: R2 ep 127 val 0.883 · คาดเสร็จ ~20:00</t>
         </is>
       </c>
     </row>
@@ -1144,21 +1146,15 @@
           <t>unlearn B4-B7 ep50 → USAI R1 → R2 Block5a-B7</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>unlearned</t>
-        </is>
-      </c>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>กำลังรัน</t>
+          <t>รอตัดสินใจ</t>
         </is>
       </c>
       <c r="I11" s="6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>200</v>
@@ -1173,7 +1169,9 @@
         <f>IFERROR((I11+K11)/(J11+L11),"")</f>
         <v/>
       </c>
-      <c r="N11" s="8" t="n"/>
+      <c r="N11" s="8" t="n">
+        <v>0.654</v>
+      </c>
       <c r="O11" s="9">
         <f>IF(D11="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C11)*(Results!$B$5:$B$50=D11)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
         <v/>
@@ -1187,10 +1185,14 @@
           <t>2026-10-02 10:49</t>
         </is>
       </c>
-      <c r="R11" s="6" t="inlineStr"/>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:10</t>
+        </is>
+      </c>
       <c r="S11" s="10" t="inlineStr">
         <is>
-          <t>~4 นาที/epoch</t>
+          <t>หยุดเอง: GPU 1 เครื่อง 29 พัดลมเสีย (93°C) — รอซ่อม / ย้าย GPU</t>
         </is>
       </c>
     </row>
@@ -1218,14 +1220,8 @@
           <t>unlearn B4-B7 ep50 → USAI R1 → R2 Block5a-B7</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>unlearned</t>
-        </is>
-      </c>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
       <c r="H12" s="6" t="inlineStr">
         <is>
           <t>ยังไม่เริ่ม</t>
@@ -1258,11 +1254,7 @@
       </c>
       <c r="Q12" s="6" t="inlineStr"/>
       <c r="R12" s="6" t="inlineStr"/>
-      <c r="S12" s="10" t="inlineStr">
-        <is>
-          <t>ต่อจาก U2 อัตโนมัติ</t>
-        </is>
-      </c>
+      <c r="S12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -3083,7 +3075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3162,11 +3154,19 @@
           <t>(1) ถ้าเข้าเครื่อง 28 ได้</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>(1) เครื่อง 28 bs 16 (หยุด llama-server ชั่วคราว)</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>รอตัดสินใจ</t>
+          <t>เสร็จ</t>
         </is>
       </c>
     </row>
@@ -3204,27 +3204,56 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>ResNet-152V2</t>
+          <t>GPU 1 เครื่อง 29 พัดลมเสีย</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ทำถ้า GPU ว่างหลัง EfficientNet-B5 เสร็จ</t>
+          <t>ซ่อม/เปลี่ยนพัดลม · ติดพัดลมเคสชั่วคราว · ส่งเคลม</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>หลัง EffNet-B5 เสร็จ</t>
+          <t>แจ้งผู้ดูแลเครื่อง</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr"/>
       <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>รอตัดสินใจ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>ResNet-152V2</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>ทำถ้า GPU ว่างหลัง EfficientNet-B5 เสร็จ</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>หลัง EffNet-B5 เสร็จ</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>ยังไม่เริ่ม</t>
         </is>
@@ -3558,41 +3587,93 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>U2</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>GPU 1 เครื่อง 29 พัดลม 0% ร้อน 93°C (shutdown 94°C) throttle เหลือ ~1/4 ความเร็ว</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>หยุด U2 ที่ R1 ep 13; ห้ามใช้ GPU 1 จนกว่าจะซ่อม (ASUS RTX 2080 Ti, PCIe 65:00.0)</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>C2 pre-train OOM บนเครื่อง 29 ที่ bs 16 และ 8 (bs 4 ได้)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>ย้ายไปเครื่อง 28 (3090 Ti) — สร้าง env unlearn26 (tf 2.6.2) ใหม่</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>d9176c7</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>เครื่อง 28: bs 16 OOM เพราะ llama-server (root, docker 9a041d11a39f) ใช้ 8 GB</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>ผู้ใช้หยุด container เอง → bs 16 ผ่าน → เริ่ม P1 15:49 · ต้อง sudo docker start 9a041d11a39f หลัง P2 เสร็จ</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>ตั้ง SSH key Mac → เครื่อง 29 (แก้ permission ~/.ssh)</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Claude เช็คสถานะเองได้</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n"/>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="4" t="n"/>
+      <c r="E17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>

</xml_diff>

<commit_message>
Tracker: unlearned seeds 2-3 running on machine 28 GPU 0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experiment_Tracker_X1X2.xlsx
+++ b/experiments/Experiment_Tracker_X1X2.xlsx
@@ -1143,18 +1143,24 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>unlearn B4-B7 ep50 → USAI R1 → R2 Block5a-B7</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="6" t="inlineStr"/>
+          <t>unlearn B4-B7 ep50 → USAI R1 → R2 Block5a-B7 · เครื่อง 28 GPU 0</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>unlearned (m28)</t>
+        </is>
+      </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>รอตัดสินใจ</t>
+          <t>กำลังรัน</t>
         </is>
       </c>
       <c r="I11" s="6" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>200</v>
@@ -1169,9 +1175,7 @@
         <f>IFERROR((I11+K11)/(J11+L11),"")</f>
         <v/>
       </c>
-      <c r="N11" s="8" t="n">
-        <v>0.654</v>
-      </c>
+      <c r="N11" s="8" t="n"/>
       <c r="O11" s="9">
         <f>IF(D11="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C11)*(Results!$B$5:$B$50=D11)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
         <v/>
@@ -1182,17 +1186,13 @@
       </c>
       <c r="Q11" s="6" t="inlineStr">
         <is>
-          <t>2026-10-02 10:49</t>
-        </is>
-      </c>
-      <c r="R11" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-02 14:10</t>
-        </is>
-      </c>
+          <t>2026-10-02 15:57</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="inlineStr"/>
       <c r="S11" s="10" t="inlineStr">
         <is>
-          <t>หยุดเอง: GPU 1 เครื่อง 29 พัดลมเสีย (93°C) — รอซ่อม / ย้าย GPU</t>
+          <t>ย้ายจาก m29 GPU 1 (พัดลมเสีย) · evaluate บน m29 หลังเสร็จ</t>
         </is>
       </c>
     </row>
@@ -1217,11 +1217,17 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>unlearn B4-B7 ep50 → USAI R1 → R2 Block5a-B7</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
+          <t>unlearn B4-B7 ep50 → USAI R1 → R2 Block5a-B7 · เครื่อง 28 GPU 0</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>unlearned (m28)</t>
+        </is>
+      </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
           <t>ยังไม่เริ่ม</t>
@@ -1254,7 +1260,11 @@
       </c>
       <c r="Q12" s="6" t="inlineStr"/>
       <c r="R12" s="6" t="inlineStr"/>
-      <c r="S12" s="10" t="inlineStr"/>
+      <c r="S12" s="10" t="inlineStr">
+        <is>
+          <t>ต่อจาก U2 อัตโนมัติ</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -3660,27 +3670,43 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>U2–U3</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>copy Traindf/Valdf จาก m29 → m28 (md5 ตรง), ภาพครบ 100% หลังแปลง path</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>เริ่ม unlearned seed 2 → 3 บน m28 GPU 0 (2080 Ti พัดลมปกติ) 15:57</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>ตั้ง SSH key Mac → เครื่อง 29 (แก้ permission ~/.ssh)</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Claude เช็คสถานะเองได้</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="4" t="n"/>
+      <c r="E18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>

</xml_diff>

<commit_message>
Tracker: status 2026-10-03 (O1 done, O2 R2 ep 87, U2 restarted on m28, C2 R1 ep 27)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experiment_Tracker_X1X2.xlsx
+++ b/experiments/Experiment_Tracker_X1X2.xlsx
@@ -594,7 +594,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2) · อัปเดต 2026-10-02 15:50</t>
+          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2) · อัปเดต 2026-10-03 15:55</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="I5" s="6" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="J5" s="4" t="n">
         <v>200</v>
@@ -753,7 +753,9 @@
         <f>IFERROR((I5+K5)/(J5+L5),"")</f>
         <v/>
       </c>
-      <c r="N5" s="8" t="n"/>
+      <c r="N5" s="8" t="n">
+        <v>0.8028</v>
+      </c>
       <c r="O5" s="9">
         <f>IF(D5="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C5)*(Results!$B$5:$B$50=D5)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
         <v/>
@@ -770,7 +772,7 @@
       <c r="R5" s="6" t="inlineStr"/>
       <c r="S5" s="10" t="inlineStr">
         <is>
-          <t>~42 นาที/epoch → R1 ≈ 5.8 วัน · เครื่อง 29 OOM (bs 16/8) จึงย้ายมาเครื่อง 28</t>
+          <t>10-03 15:51: ep 27/200 · ~53 นาที/epoch ช่วงที่ U2 รันคู่ → R1 ≈ 8 ต.ค.</t>
         </is>
       </c>
     </row>
@@ -940,7 +942,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>กำลังรัน</t>
+          <t>เสร็จ</t>
         </is>
       </c>
       <c r="I8" s="6" t="n">
@@ -950,7 +952,7 @@
         <v>200</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>127</v>
+        <v>200</v>
       </c>
       <c r="L8" s="6" t="n">
         <v>200</v>
@@ -960,7 +962,7 @@
         <v/>
       </c>
       <c r="N8" s="8" t="n">
-        <v>0.883</v>
+        <v>0.8811</v>
       </c>
       <c r="O8" s="9">
         <f>IF(D8="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C8)*(Results!$B$5:$B$50=D8)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
@@ -975,10 +977,14 @@
           <t>2026-10-01 16:43</t>
         </is>
       </c>
-      <c r="R8" s="6" t="inlineStr"/>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="S8" s="10" t="inlineStr">
         <is>
-          <t>10-02 15:00: R2 ep 127 val 0.883 · คาดเสร็จ ~20:00</t>
+          <t>R2 val 0.8811 · กำลัง evaluate (CPU, screen eval_o1)</t>
         </is>
       </c>
     </row>
@@ -1016,17 +1022,17 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>ยังไม่เริ่ม</t>
+          <t>กำลังรัน</t>
         </is>
       </c>
       <c r="I9" s="6" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>200</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>200</v>
@@ -1035,7 +1041,9 @@
         <f>IFERROR((I9+K9)/(J9+L9),"")</f>
         <v/>
       </c>
-      <c r="N9" s="8" t="n"/>
+      <c r="N9" s="8" t="n">
+        <v>0.878</v>
+      </c>
       <c r="O9" s="9">
         <f>IF(D9="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C9)*(Results!$B$5:$B$50=D9)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
         <v/>
@@ -1044,11 +1052,15 @@
         <f>IF(D9="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C9)*(Results!$B$5:$B$50=D9)*(Results!$C$5:$C$50="field"),0),0))),""))</f>
         <v/>
       </c>
-      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="R9" s="6" t="inlineStr"/>
       <c r="S9" s="10" t="inlineStr">
         <is>
-          <t>ต่อจาก O1 อัตโนมัติ</t>
+          <t>10-03 15:51: R2 ep 87 · คาดเสร็จ ~4 ต.ค. เช้า</t>
         </is>
       </c>
     </row>
@@ -1186,13 +1198,13 @@
       </c>
       <c r="Q11" s="6" t="inlineStr">
         <is>
-          <t>2026-10-02 15:57</t>
+          <t>2026-10-03 15:52</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr"/>
       <c r="S11" s="10" t="inlineStr">
         <is>
-          <t>ย้ายจาก m29 GPU 1 (พัดลมเสีย) · evaluate บน m29 หลังเสร็จ</t>
+          <t>รอบแรก (10-02 15:57) หยุดที่ ep 7 ตอน 16:23 น่าจะ RAM เต็ม (m28 RAM 31 GB) → เริ่มใหม่</t>
         </is>
       </c>
     </row>
@@ -3688,39 +3700,71 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>unlearned seed 2 บน m28 หยุดเอง 10-02 16:23 (ep 7, ไม่มี error, screen หาย) — น่าจะ RAM เต็มตอนรัน A1 คู่กับ C2</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>เริ่มใหม่ 10-03 15:52; ห้ามรันงานวิเคราะห์หนักบน m28</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>A1–A3</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>A1 face metrics, A2 ultrasound stats, A3 flip consistency เสร็จ</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>ข้อความแก้ paper: experiments/paper_revision/Revision_A1-A5.md</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>ตั้ง SSH key Mac → เครื่อง 29 (แก้ permission ~/.ssh)</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>Claude เช็คสถานะเองได้</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="4" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n"/>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="4" t="n"/>
+      <c r="E20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>

</xml_diff>

<commit_message>
Tracker: power outage 10-05, all stages resumed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experiment_Tracker_X1X2.xlsx
+++ b/experiments/Experiment_Tracker_X1X2.xlsx
@@ -594,7 +594,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2) · อัปเดต 2026-10-03 15:55</t>
+          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2) · อัปเดต 2026-10-05 10:20</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="I5" s="6" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="J5" s="4" t="n">
         <v>200</v>
@@ -754,7 +754,7 @@
         <v/>
       </c>
       <c r="N5" s="8" t="n">
-        <v>0.8028</v>
+        <v>0.8048</v>
       </c>
       <c r="O5" s="9">
         <f>IF(D5="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C5)*(Results!$B$5:$B$50=D5)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
@@ -772,7 +772,7 @@
       <c r="R5" s="6" t="inlineStr"/>
       <c r="S5" s="10" t="inlineStr">
         <is>
-          <t>10-03 15:51: ep 27/200 · ~53 นาที/epoch ช่วงที่ U2 รันคู่ → R1 ≈ 8 ต.ค.</t>
+          <t>10-05 ไฟดับที่ ep 45 → resume 10:14 อีก 156 ep (~43 นาที/ep) → R1 ≈ 10 ต.ค.</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>กำลังรัน</t>
+          <t>เสร็จ</t>
         </is>
       </c>
       <c r="I9" s="6" t="n">
@@ -1032,7 +1032,7 @@
         <v>200</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>87</v>
+        <v>200</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>200</v>
@@ -1042,7 +1042,7 @@
         <v/>
       </c>
       <c r="N9" s="8" t="n">
-        <v>0.878</v>
+        <v>0.875</v>
       </c>
       <c r="O9" s="9">
         <f>IF(D9="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C9)*(Results!$B$5:$B$50=D9)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
@@ -1057,10 +1057,14 @@
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="R9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
       <c r="S9" s="10" t="inlineStr">
         <is>
-          <t>10-03 15:51: R2 ep 87 · คาดเสร็จ ~4 ต.ค. เช้า</t>
+          <t>R2 val 0.875 · evaluate (CPU, screen eval_o2)</t>
         </is>
       </c>
     </row>
@@ -1093,16 +1097,16 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>original</t>
+          <t>run_gpu0</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>ยังไม่เริ่ม</t>
+          <t>กำลังรัน</t>
         </is>
       </c>
       <c r="I10" s="6" t="n">
-        <v>0</v>
+        <v>153</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>200</v>
@@ -1117,7 +1121,9 @@
         <f>IFERROR((I10+K10)/(J10+L10),"")</f>
         <v/>
       </c>
-      <c r="N10" s="8" t="n"/>
+      <c r="N10" s="8" t="n">
+        <v>0.7088</v>
+      </c>
       <c r="O10" s="9">
         <f>IF(D10="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C10)*(Results!$B$5:$B$50=D10)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
         <v/>
@@ -1126,11 +1132,15 @@
         <f>IF(D10="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C10)*(Results!$B$5:$B$50=D10)*(Results!$C$5:$C$50="field"),0),0))),""))</f>
         <v/>
       </c>
-      <c r="Q10" s="6" t="inlineStr"/>
+      <c r="Q10" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
       <c r="R10" s="6" t="inlineStr"/>
       <c r="S10" s="10" t="inlineStr">
         <is>
-          <t>ต่อจาก O2 อัตโนมัติ</t>
+          <t>10-05 ไฟดับที่ R1 ep 154 → resume 10:14 อีก 47 ep → R2 → eval อัตโนมัติ</t>
         </is>
       </c>
     </row>
@@ -1172,13 +1182,13 @@
         </is>
       </c>
       <c r="I11" s="6" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>200</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>200</v>
@@ -1187,7 +1197,9 @@
         <f>IFERROR((I11+K11)/(J11+L11),"")</f>
         <v/>
       </c>
-      <c r="N11" s="8" t="n"/>
+      <c r="N11" s="8" t="n">
+        <v>0.8826000000000001</v>
+      </c>
       <c r="O11" s="9">
         <f>IF(D11="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C11)*(Results!$B$5:$B$50=D11)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
         <v/>
@@ -1204,7 +1216,7 @@
       <c r="R11" s="6" t="inlineStr"/>
       <c r="S11" s="10" t="inlineStr">
         <is>
-          <t>รอบแรก (10-02 15:57) หยุดที่ ep 7 ตอน 16:23 น่าจะ RAM เต็ม (m28 RAM 31 GB) → เริ่มใหม่</t>
+          <t>R1 val 0.660 · 10-05 ไฟดับที่ R2 ep 42 → resume 10:14 อีก 159 ep → ต่อ U3</t>
         </is>
       </c>
     </row>
@@ -3723,22 +3735,22 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>A1–A3</t>
+          <t>O3, U2, P1</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>A1 face metrics, A2 ultrasound stats, A3 flip consistency เสร็จ</t>
+          <t>ไฟดับ ทั้งเครื่อง 28 และ 29 รีบูต (~10:05) screen หายหมด</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>ข้อความแก้ paper: experiments/paper_revision/Revision_A1-A5.md</t>
+          <t>เพิ่ม experiments/resume.sh: ต่อจาก checkpoint ล่าสุด เทรนเฉพาะ epoch ที่เหลือ (เสีย epoch ที่ค้างอยู่ 1 epoch/งาน) · optimizer state เริ่มใหม่ตอน resume</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
@@ -3746,32 +3758,48 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>A1–A3</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>A1 face metrics, A2 ultrasound stats, A3 flip consistency เสร็จ</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>ข้อความแก้ paper: experiments/paper_revision/Revision_A1-A5.md</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>ตั้ง SSH key Mac → เครื่อง 29 (แก้ permission ~/.ssh)</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Claude เช็คสถานะเองได้</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="4" t="n"/>
+      <c r="E21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>

</xml_diff>

<commit_message>
Tracker: X2 original done, unlearned seed 2 evaluated, C1 queue started (600 ep)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experiment_Tracker_X1X2.xlsx
+++ b/experiments/Experiment_Tracker_X1X2.xlsx
@@ -594,7 +594,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2) · อัปเดต 2026-10-05 10:20</t>
+          <t>Experiment Tracker — X1 / X2 (EfficientNet-B5) · เครื่อง 29 (RTX 2080 Ti ×2, env AI tf 2.6.2) · อัปเดต 2026-10-06 10:50</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="I5" s="6" t="n">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="J5" s="4" t="n">
         <v>200</v>
@@ -754,7 +754,7 @@
         <v/>
       </c>
       <c r="N5" s="8" t="n">
-        <v>0.8048</v>
+        <v>0.8282</v>
       </c>
       <c r="O5" s="9">
         <f>IF(D5="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C5)*(Results!$B$5:$B$50=D5)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
@@ -772,7 +772,7 @@
       <c r="R5" s="6" t="inlineStr"/>
       <c r="S5" s="10" t="inlineStr">
         <is>
-          <t>10-05 ไฟดับที่ ep 45 → resume 10:14 อีก 156 ep (~43 นาที/ep) → R1 ≈ 10 ต.ค.</t>
+          <t>10-06 10:41: ep 70/200 (~57 นาที/ep) → R1 ≈ 11 ต.ค.</t>
         </is>
       </c>
     </row>
@@ -1102,17 +1102,17 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>กำลังรัน</t>
+          <t>เสร็จ</t>
         </is>
       </c>
       <c r="I10" s="6" t="n">
-        <v>153</v>
+        <v>200</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>200</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="L10" s="6" t="n">
         <v>200</v>
@@ -1122,7 +1122,7 @@
         <v/>
       </c>
       <c r="N10" s="8" t="n">
-        <v>0.7088</v>
+        <v>0.8811</v>
       </c>
       <c r="O10" s="9">
         <f>IF(D10="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C10)*(Results!$B$5:$B$50=D10)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
@@ -1137,10 +1137,14 @@
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="R10" s="6" t="inlineStr"/>
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="S10" s="10" t="inlineStr">
         <is>
-          <t>10-05 ไฟดับที่ R1 ep 154 → resume 10:14 อีก 47 ep → R2 → eval อัตโนมัติ</t>
+          <t>R1 resume หลังไฟดับ</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1182,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>กำลังรัน</t>
+          <t>เสร็จ</t>
         </is>
       </c>
       <c r="I11" s="6" t="n">
@@ -1188,7 +1192,7 @@
         <v>200</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>41</v>
+        <v>200</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>200</v>
@@ -1198,7 +1202,7 @@
         <v/>
       </c>
       <c r="N11" s="8" t="n">
-        <v>0.8826000000000001</v>
+        <v>0.8948</v>
       </c>
       <c r="O11" s="9">
         <f>IF(D11="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C11)*(Results!$B$5:$B$50=D11)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
@@ -1213,10 +1217,14 @@
           <t>2026-10-03 15:52</t>
         </is>
       </c>
-      <c r="R11" s="6" t="inlineStr"/>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="S11" s="10" t="inlineStr">
         <is>
-          <t>R1 val 0.660 · 10-05 ไฟดับที่ R2 ep 42 → resume 10:14 อีก 159 ep → ต่อ U3</t>
+          <t>R2 resume หลังไฟดับ · evaluate บน m29 (copy โมเดล md5 ตรง)</t>
         </is>
       </c>
     </row>
@@ -1254,11 +1262,11 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>ยังไม่เริ่ม</t>
+          <t>กำลังรัน</t>
         </is>
       </c>
       <c r="I12" s="6" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>200</v>
@@ -1273,7 +1281,9 @@
         <f>IFERROR((I12+K12)/(J12+L12),"")</f>
         <v/>
       </c>
-      <c r="N12" s="8" t="n"/>
+      <c r="N12" s="8" t="n">
+        <v>0.657</v>
+      </c>
       <c r="O12" s="9">
         <f>IF(D12="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C12)*(Results!$B$5:$B$50=D12)*(Results!$C$5:$C$50="lab"),0),0))),""))</f>
         <v/>
@@ -1282,11 +1292,15 @@
         <f>IF(D12="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C12)*(Results!$B$5:$B$50=D12)*(Results!$C$5:$C$50="field"),0),0))),""))</f>
         <v/>
       </c>
-      <c r="Q12" s="6" t="inlineStr"/>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="R12" s="6" t="inlineStr"/>
       <c r="S12" s="10" t="inlineStr">
         <is>
-          <t>ต่อจาก U2 อัตโนมัติ</t>
+          <t>คาดเสร็จ ~7 ต.ค.</t>
         </is>
       </c>
     </row>
@@ -1311,14 +1325,20 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>original pipeline, R2 ยาวขึ้น (compute-matched)</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr"/>
-      <c r="G13" s="6" t="inlineStr"/>
+          <t>original pipeline, R2 = 600 ep (compute-matched, capped)</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>queue_gpu0 (m29)</t>
+        </is>
+      </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>รอตัดสินใจ</t>
+          <t>กำลังรัน</t>
         </is>
       </c>
       <c r="I13" s="6" t="n">
@@ -1330,7 +1350,9 @@
       <c r="K13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="6" t="n"/>
+      <c r="L13" s="6" t="n">
+        <v>600</v>
+      </c>
       <c r="M13" s="7">
         <f>IFERROR((I13+K13)/(J13+L13),"")</f>
         <v/>
@@ -1344,11 +1366,15 @@
         <f>IF(D13="","",IFERROR(1/(1/INDEX(Results!$D$5:$D$50,MATCH(1,INDEX((Results!$A$5:$A$50=C13)*(Results!$B$5:$B$50=D13)*(Results!$C$5:$C$50="field"),0),0))),""))</f>
         <v/>
       </c>
-      <c r="Q13" s="6" t="inlineStr"/>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-06 10:46</t>
+        </is>
+      </c>
       <c r="R13" s="6" t="inlineStr"/>
       <c r="S13" s="10" t="inlineStr">
         <is>
-          <t>รอ D2 → R2 ep total = E_C1</t>
+          <t>queue m29 GPU 0 · ~2.3 วัน/seed · eval อัตโนมัติ</t>
         </is>
       </c>
     </row>
@@ -1373,14 +1399,20 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>original pipeline, R2 ยาวขึ้น (compute-matched)</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr"/>
+          <t>original pipeline, R2 = 600 ep (compute-matched, capped)</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>queue_gpu0 (m29)</t>
+        </is>
+      </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>รอตัดสินใจ</t>
+          <t>ยังไม่เริ่ม</t>
         </is>
       </c>
       <c r="I14" s="6" t="n">
@@ -1392,7 +1424,9 @@
       <c r="K14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="L14" s="6" t="n"/>
+      <c r="L14" s="6" t="n">
+        <v>600</v>
+      </c>
       <c r="M14" s="7">
         <f>IFERROR((I14+K14)/(J14+L14),"")</f>
         <v/>
@@ -1408,7 +1442,11 @@
       </c>
       <c r="Q14" s="6" t="inlineStr"/>
       <c r="R14" s="6" t="inlineStr"/>
-      <c r="S14" s="10" t="inlineStr"/>
+      <c r="S14" s="10" t="inlineStr">
+        <is>
+          <t>queue m29 GPU 0 · ~2.3 วัน/seed · eval อัตโนมัติ</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1431,14 +1469,20 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>original pipeline, R2 ยาวขึ้น (compute-matched)</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr"/>
-      <c r="G15" s="6" t="inlineStr"/>
+          <t>original pipeline, R2 = 600 ep (compute-matched, capped)</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>queue_gpu0 (m29)</t>
+        </is>
+      </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>รอตัดสินใจ</t>
+          <t>ยังไม่เริ่ม</t>
         </is>
       </c>
       <c r="I15" s="6" t="n">
@@ -1450,7 +1494,9 @@
       <c r="K15" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="L15" s="6" t="n"/>
+      <c r="L15" s="6" t="n">
+        <v>600</v>
+      </c>
       <c r="M15" s="7">
         <f>IFERROR((I15+K15)/(J15+L15),"")</f>
         <v/>
@@ -1466,7 +1512,11 @@
       </c>
       <c r="Q15" s="6" t="inlineStr"/>
       <c r="R15" s="6" t="inlineStr"/>
-      <c r="S15" s="10" t="inlineStr"/>
+      <c r="S15" s="10" t="inlineStr">
+        <is>
+          <t>queue m29 GPU 0 · ~2.3 วัน/seed · eval อัตโนมัติ</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -3212,7 +3262,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>วิธี compute-match ของ C1</t>
+          <t>วิธี compute-match ของ C1 (ตัดสินแล้ว: cap 600 ep, 10-06)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -3735,22 +3785,22 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>O3, U2, P1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>ไฟดับ ทั้งเครื่อง 28 และ 29 รีบูต (~10:05) screen หายหมด</t>
+          <t>ตั้ง E_C1 = 600 (cap) และเริ่มคิว C1 seed 1→2→3 บน m29 GPU 0 (queue.sh)</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>เพิ่ม experiments/resume.sh: ต่อจาก checkpoint ล่าสุด เทรนเฉพาะ epoch ที่เหลือ (เสีย epoch ที่ค้างอยู่ 1 epoch/งาน) · optimizer state เริ่มใหม่ตอน resume</t>
+          <t>ผล X2 ตอนนี้: lab acc เท่ากัน, macro-F1 unlearned สูงกว่า ~0.015 ทุก seed; field acc ของ unlearned seed 2 (0.736) ไม่ซ้ำ seed 1 (0.849)</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
@@ -3758,22 +3808,22 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>A1–A3</t>
+          <t>O3, U2, P1</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>A1 face metrics, A2 ultrasound stats, A3 flip consistency เสร็จ</t>
+          <t>ไฟดับ ทั้งเครื่อง 28 และ 29 รีบูต (~10:05) screen หายหมด</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>ข้อความแก้ paper: experiments/paper_revision/Revision_A1-A5.md</t>
+          <t>เพิ่ม experiments/resume.sh: ต่อจาก checkpoint ล่าสุด เทรนเฉพาะ epoch ที่เหลือ (เสีย epoch ที่ค้างอยู่ 1 epoch/งาน) · optimizer state เริ่มใหม่ตอน resume</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr"/>
@@ -3781,32 +3831,48 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>A1–A3</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>A1 face metrics, A2 ultrasound stats, A3 flip consistency เสร็จ</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>ข้อความแก้ paper: experiments/paper_revision/Revision_A1-A5.md</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>ตั้ง SSH key Mac → เครื่อง 29 (แก้ permission ~/.ssh)</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Claude เช็คสถานะเองได้</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="4" t="n"/>
+      <c r="E22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>

</xml_diff>